<commit_message>
Locator changes fixed and test data updated for HRM
Locator changes fixed and test data updated for HRM
</commit_message>
<xml_diff>
--- a/testdata/EmpDetailsMigrationData.xlsx
+++ b/testdata/EmpDetailsMigrationData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920"/>
+    <workbookView windowWidth="13860" windowHeight="6920"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
   <si>
     <t>Emp. ID</t>
   </si>
@@ -51,9 +51,6 @@
   </si>
   <si>
     <t>104</t>
-  </si>
-  <si>
-    <t>GWP0053</t>
   </si>
   <si>
     <t>GWP0054</t>
@@ -1245,8 +1242,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="3"/>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
@@ -1290,24 +1287,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" location="EMP_SHIFT_TYPE#,00001,00001" display="GWP0053"/>
-    <hyperlink ref="A4" r:id="rId1" location="EMP_SHIFT_TYPE#,00001,00001" display="GWP0054"/>
+    <hyperlink ref="A3" r:id="rId1" location="EMP_SHIFT_TYPE#,00001,00001" display="GWP0054"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>